<commit_message>
Confirmation of Order is error free
</commit_message>
<xml_diff>
--- a/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
+++ b/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="0" windowWidth="16572" windowHeight="6384"/>
+    <workbookView xWindow="3252" yWindow="0" windowWidth="16572" windowHeight="6384"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -146,9 +146,6 @@
     <t>LiveOnly@ttstrain.com</t>
   </si>
   <si>
-    <t>UpcomingNoConnInfo.com</t>
-  </si>
-  <si>
     <t>RecordedOnly@ttstrain.com</t>
   </si>
   <si>
@@ -167,9 +164,6 @@
     <t>LivePlusOnDemand</t>
   </si>
   <si>
-    <t>UpcomingHasConnInfo.com</t>
-  </si>
-  <si>
     <t>LiveOnlyHasConnectionInfo@ttstrain.com</t>
   </si>
   <si>
@@ -192,6 +186,12 @@
   </si>
   <si>
     <t>OnDemandOnly</t>
+  </si>
+  <si>
+    <t>UpcomingNoConnInfo</t>
+  </si>
+  <si>
+    <t>UpcomingHasConnInfo</t>
   </si>
 </sst>
 </file>
@@ -523,6 +523,7 @@
   <dimension ref="A1:Y15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
     <col min="7" max="7" width="25.88671875" customWidth="1"/>
     <col min="10" max="10" width="38.6640625" customWidth="1"/>
   </cols>
@@ -621,10 +622,10 @@
         <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H2" t="s">
         <v>27</v>
@@ -668,10 +669,10 @@
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H3" t="s">
         <v>27</v>
@@ -680,7 +681,7 @@
         <v>28</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K3" t="s">
         <v>29</v>
@@ -715,10 +716,10 @@
         <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H4" t="s">
         <v>27</v>
@@ -765,10 +766,10 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
         <v>27</v>
@@ -815,10 +816,10 @@
         <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H6" t="s">
         <v>27</v>
@@ -865,10 +866,10 @@
         <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s">
         <v>27</v>
@@ -877,7 +878,7 @@
         <v>28</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K8" t="s">
         <v>29</v>
@@ -912,10 +913,10 @@
         <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>27</v>
@@ -924,7 +925,7 @@
         <v>28</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s">
         <v>29</v>
@@ -959,10 +960,10 @@
         <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="H10" t="s">
         <v>27</v>
@@ -971,7 +972,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K10" t="s">
         <v>29</v>
@@ -1009,10 +1010,10 @@
         <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="H11" t="s">
         <v>27</v>
@@ -1021,7 +1022,7 @@
         <v>28</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K11" t="s">
         <v>29</v>
@@ -1059,10 +1060,10 @@
         <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G12" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="H12" t="s">
         <v>27</v>
@@ -1071,7 +1072,7 @@
         <v>28</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K12" t="s">
         <v>29</v>
@@ -1106,10 +1107,10 @@
         <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H14" t="s">
         <v>27</v>
@@ -1153,10 +1154,10 @@
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H15" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
checkpoint for formatting Confirmation message
</commit_message>
<xml_diff>
--- a/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
+++ b/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="3252" yWindow="0" windowWidth="16572" windowHeight="6384"/>
+    <workbookView xWindow="4224" yWindow="0" windowWidth="16572" windowHeight="6384"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -128,27 +128,6 @@
     <t>USA</t>
   </si>
   <si>
-    <t>CDRom@UpcomingNoConnInfo.com</t>
-  </si>
-  <si>
-    <t>LivePlusOnDemand@UpcomingNoConnInfo.com</t>
-  </si>
-  <si>
-    <t>Premier@UpcomingNoConnInfo.com</t>
-  </si>
-  <si>
-    <t>OnDemandOnly@Recorded.com</t>
-  </si>
-  <si>
-    <t>CDRom@Recorded.com</t>
-  </si>
-  <si>
-    <t>LiveOnly@ttstrain.com</t>
-  </si>
-  <si>
-    <t>RecordedOnly@ttstrain.com</t>
-  </si>
-  <si>
     <t>LiveOnly</t>
   </si>
   <si>
@@ -164,21 +143,6 @@
     <t>LivePlusOnDemand</t>
   </si>
   <si>
-    <t>LiveOnlyHasConnectionInfo@ttstrain.com</t>
-  </si>
-  <si>
-    <t>RecordedOnlyHasConnectionInfo@ttstrain.com</t>
-  </si>
-  <si>
-    <t>CDRomHasConnectionInfo@ttstrain.com</t>
-  </si>
-  <si>
-    <t>LivePlusOnDemandHasConnectionInfo@ttstrain.com</t>
-  </si>
-  <si>
-    <t>PremierHasConnectionInfo@ttstrain.com</t>
-  </si>
-  <si>
     <t>Recorded</t>
   </si>
   <si>
@@ -192,6 +156,42 @@
   </si>
   <si>
     <t>UpcomingHasConnInfo</t>
+  </si>
+  <si>
+    <t>LiveOnly@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>RecordedOnly@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>CDRom@UpcomingNoConnInfo1.com</t>
+  </si>
+  <si>
+    <t>LivePlusOnDemand@UpcomingNoConnInfo1.com</t>
+  </si>
+  <si>
+    <t>Premier@UpcomingNoConnInfo1.com</t>
+  </si>
+  <si>
+    <t>LiveOnlyHasConnectionInfo@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>RecordedOnlyHasConnectionInfo@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>CDRomHasConnectionInfo@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>LivePlusOnDemandHasConnectionInfo@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>PremierHasConnectionInfo@ttstrain1.com</t>
+  </si>
+  <si>
+    <t>OnDemandOnly@Recorded1.com</t>
+  </si>
+  <si>
+    <t>CDRom@Recorded1.com</t>
   </si>
 </sst>
 </file>
@@ -622,10 +622,10 @@
         <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
         <v>27</v>
@@ -634,7 +634,7 @@
         <v>28</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="K2" t="s">
         <v>29</v>
@@ -669,10 +669,10 @@
         <v>19</v>
       </c>
       <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
         <v>42</v>
-      </c>
-      <c r="G3" t="s">
-        <v>54</v>
       </c>
       <c r="H3" t="s">
         <v>27</v>
@@ -681,7 +681,7 @@
         <v>28</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K3" t="s">
         <v>29</v>
@@ -716,10 +716,10 @@
         <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
         <v>27</v>
@@ -728,7 +728,7 @@
         <v>28</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K4" t="s">
         <v>29</v>
@@ -766,10 +766,10 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
         <v>27</v>
@@ -778,7 +778,7 @@
         <v>28</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="K5" t="s">
         <v>29</v>
@@ -816,10 +816,10 @@
         <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
         <v>27</v>
@@ -828,7 +828,7 @@
         <v>28</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
         <v>29</v>
@@ -866,10 +866,10 @@
         <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="H8" t="s">
         <v>27</v>
@@ -878,7 +878,7 @@
         <v>28</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K8" t="s">
         <v>29</v>
@@ -913,10 +913,10 @@
         <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s">
         <v>27</v>
@@ -925,7 +925,7 @@
         <v>28</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K9" t="s">
         <v>29</v>
@@ -960,10 +960,10 @@
         <v>19</v>
       </c>
       <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
         <v>43</v>
-      </c>
-      <c r="G10" t="s">
-        <v>55</v>
       </c>
       <c r="H10" t="s">
         <v>27</v>
@@ -972,7 +972,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="K10" t="s">
         <v>29</v>
@@ -1010,10 +1010,10 @@
         <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="H11" t="s">
         <v>27</v>
@@ -1022,7 +1022,7 @@
         <v>28</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K11" t="s">
         <v>29</v>
@@ -1060,10 +1060,10 @@
         <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="H12" t="s">
         <v>27</v>
@@ -1072,7 +1072,7 @@
         <v>28</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="K12" t="s">
         <v>29</v>
@@ -1107,10 +1107,10 @@
         <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="H14" t="s">
         <v>27</v>
@@ -1119,7 +1119,7 @@
         <v>28</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="K14" t="s">
         <v>29</v>
@@ -1154,10 +1154,10 @@
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="H15" t="s">
         <v>27</v>
@@ -1166,7 +1166,7 @@
         <v>28</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="K15" t="s">
         <v>29</v>
@@ -1189,18 +1189,18 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1"/>
-    <hyperlink ref="J3" r:id="rId2"/>
-    <hyperlink ref="J4" r:id="rId3"/>
+    <hyperlink ref="J2" r:id="rId1" display="LiveOnly@ttstrain.com"/>
+    <hyperlink ref="J3" r:id="rId2" display="RecordedOnly@ttstrain.com"/>
+    <hyperlink ref="J4" r:id="rId3" display="CDRom@UpcomingNoConnInfo.com"/>
     <hyperlink ref="J5" r:id="rId4" display="LivePlusOnDemand@UpcomingHasConnInfo.com"/>
     <hyperlink ref="J6" r:id="rId5" display="Premier@UpcomingHasConnInfo.com"/>
-    <hyperlink ref="J14" r:id="rId6"/>
-    <hyperlink ref="J15" r:id="rId7"/>
-    <hyperlink ref="J8" r:id="rId8"/>
-    <hyperlink ref="J9" r:id="rId9"/>
-    <hyperlink ref="J10" r:id="rId10"/>
-    <hyperlink ref="J11" r:id="rId11"/>
-    <hyperlink ref="J12" r:id="rId12"/>
+    <hyperlink ref="J14" r:id="rId6" display="OnDemandOnly@Recorded.com"/>
+    <hyperlink ref="J15" r:id="rId7" display="CDRom@Recorded.com"/>
+    <hyperlink ref="J8" r:id="rId8" display="LiveOnlyHasConnectionInfo@ttstrain.com"/>
+    <hyperlink ref="J9" r:id="rId9" display="RecordedOnlyHasConnectionInfo@ttstrain.com"/>
+    <hyperlink ref="J10" r:id="rId10" display="CDRomHasConnectionInfo@ttstrain.com"/>
+    <hyperlink ref="J11" r:id="rId11" display="LivePlusOnDemandHasConnectionInfo@ttstrain.com"/>
+    <hyperlink ref="J12" r:id="rId12" display="PremierHasConnectionInfo@ttstrain.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates SQLSeeding with new versions of dbs and scripts that represent clean starting points of Production and Test versions of both dbs.
Add Excel workbook that imports sample data.
</commit_message>
<xml_diff>
--- a/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
+++ b/CUWebinars.Web/App_Data/Orders/SampleData.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\users\steve\source\repos\bankwebinars\cuwebinars.web\app_data\orders\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="5220" yWindow="0" windowWidth="16572" windowHeight="6384"/>
+    <workbookView xWindow="6216" yWindow="0" windowWidth="16572" windowHeight="6384"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -457,6 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>